<commit_message>
feat(saisatwik): publish K04 workbook blog + mark published rows in plan
- K04 "SAP EPPM Implementation Roadmap" (#5376) — traffic-intent knowledge
  blog per SAISATWIK_BLOG_PUBLISHING.md + workbook Read Me house style
  (plain, no em dashes, no filler). 3 tables, 5-question FAQ, 4 outbound
  authority (SAP.com, PMI, Standish), 6 internal incl. service-page CTA.
  8th spoke in the SAP EPPM cluster; hub #5302 re-pushed to link down to it.
- SAP-EPPM-PS-Blog-Keyword-Plan.xlsx: added Status + Live URL columns to
  Knowledge + Leads sheets; green-highlighted the 5 published rows
  (K01 -> #5302, K02 -> #5352, K03 -> #5371, K04 -> #5376,
  K65 -> #5308 Saudi Vision 2030), rest marked Pending.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SAP-EPPM-PS-Blog-Keyword-Plan.xlsx
+++ b/SAP-EPPM-PS-Blog-Keyword-Plan.xlsx
@@ -25,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -77,8 +77,19 @@
       <color rgb="0041506B"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+    </font>
+    <font>
+      <color rgb="FF006100"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FF006100"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -98,6 +109,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF375623"/>
+        <bgColor rgb="FF375623"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -127,7 +150,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -161,6 +184,15 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -534,7 +566,6 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr"/>
       <c r="B1" s="1" t="inlineStr">
         <is>
           <t>SAP EPPM / PS Blog Topic &amp; Keyword Plan</t>
@@ -542,7 +573,6 @@
       </c>
     </row>
     <row r="2" ht="32" customHeight="1">
-      <c r="A2" t="inlineStr"/>
       <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Built for Spanbix / STPL. Target geos: Middle East (UAE, KSA, Qatar, Oman, Kuwait, Bahrain), Jordan, Singapore, plus wider APAC.</t>
@@ -550,11 +580,9 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
       <c r="B3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
       <c r="B4" s="4" t="inlineStr">
         <is>
           <t>How the plan is split</t>
@@ -562,7 +590,6 @@
       </c>
     </row>
     <row r="5" ht="52" customHeight="1">
-      <c r="A5" t="inlineStr"/>
       <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Knowledge Blogs tab: top-of-funnel, informational. Built to pull organic search traffic, rank for definitions, how-to and comparison queries, build topical authority. Mostly geo-neutral because these queries are searched worldwide. This is your traffic engine.</t>
@@ -570,7 +597,6 @@
       </c>
     </row>
     <row r="6" ht="48" customHeight="1">
-      <c r="A6" t="inlineStr"/>
       <c r="B6" s="3" t="inlineStr">
         <is>
           <t>Leads Blogs tab: bottom-of-funnel, commercial and transactional. Built to capture buyers who are ready to hire an implementation partner. Heavily geo-localised because commercial SAP searches are location-based. This is your lead engine.</t>
@@ -578,7 +604,6 @@
       </c>
     </row>
     <row r="7" ht="34" customHeight="1">
-      <c r="A7" t="inlineStr"/>
       <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Industry x Product Matrix tab: the vertical angles from your MarketHub, mapped to modules. Use it to generate more titles.</t>
@@ -586,7 +611,6 @@
       </c>
     </row>
     <row r="8" ht="34" customHeight="1">
-      <c r="A8" t="inlineStr"/>
       <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Geo Keyword Bank tab: modifier lists. Combine a base keyword with a geo modifier to spin up localised variants at scale.</t>
@@ -594,11 +618,9 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
       <c r="B9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
       <c r="B10" s="4" t="inlineStr">
         <is>
           <t>How to use it</t>
@@ -606,7 +628,6 @@
       </c>
     </row>
     <row r="11" ht="48" customHeight="1">
-      <c r="A11" t="inlineStr"/>
       <c r="B11" s="3" t="inlineStr">
         <is>
           <t>1. Validate volume before committing. These are keyword targets chosen by buyer intent and competition logic, not pulled from a live tool. Run each Primary Keyword through Ahrefs, Semrush, or Google Keyword Planner (set location to your target country) to confirm volume and difficulty.</t>
@@ -614,7 +635,6 @@
       </c>
     </row>
     <row r="12" ht="34" customHeight="1">
-      <c r="A12" t="inlineStr"/>
       <c r="B12" s="3" t="inlineStr">
         <is>
           <t>2. Publish Knowledge blogs first to build authority and internal links, then point them at your Leads blogs and service pages.</t>
@@ -622,7 +642,6 @@
       </c>
     </row>
     <row r="13" ht="34" customHeight="1">
-      <c r="A13" t="inlineStr"/>
       <c r="B13" s="3" t="inlineStr">
         <is>
           <t>3. For Leads blogs, create one page per country rather than stuffing many geos into one post. Google ranks local intent better with dedicated pages.</t>
@@ -630,7 +649,6 @@
       </c>
     </row>
     <row r="14" ht="34" customHeight="1">
-      <c r="A14" t="inlineStr"/>
       <c r="B14" s="3" t="inlineStr">
         <is>
           <t>4. Priority column: 1 = build first (strong intent or strong traffic), 2 = second wave, 3 = long tail / fill.</t>
@@ -638,11 +656,9 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr"/>
       <c r="B15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
       <c r="B16" s="4" t="inlineStr">
         <is>
           <t>Note on writing</t>
@@ -650,7 +666,6 @@
       </c>
     </row>
     <row r="17" ht="48" customHeight="1">
-      <c r="A17" t="inlineStr"/>
       <c r="B17" s="3" t="inlineStr">
         <is>
           <t>Keep the house style: plain, direct, no em dashes, no filler words like seamless, powerful, ecosystem. Lead every Leads blog with the business outcome, not the module.</t>
@@ -668,7 +683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H68"/>
+  <dimension ref="A1:J68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -679,6 +694,8 @@
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -722,165 +739,215 @@
           <t>Priority</t>
         </is>
       </c>
+      <c r="I1" s="15" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="J1" s="15" t="inlineStr">
+        <is>
+          <t>Live URL</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="16" t="inlineStr">
         <is>
           <t>K01</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="B2" s="16" t="inlineStr">
         <is>
           <t>EPPM</t>
         </is>
       </c>
-      <c r="C2" s="7" t="inlineStr">
+      <c r="C2" s="17" t="inlineStr">
         <is>
           <t>What is SAP EPPM? A complete guide</t>
         </is>
       </c>
-      <c r="D2" s="7" t="inlineStr">
+      <c r="D2" s="17" t="inlineStr">
         <is>
           <t>what is SAP EPPM</t>
         </is>
       </c>
-      <c r="E2" s="7" t="inlineStr">
+      <c r="E2" s="17" t="inlineStr">
         <is>
           <t>SAP EPPM meaning, SAP EPPM full form, enterprise portfolio project management</t>
         </is>
       </c>
-      <c r="F2" s="6" t="inlineStr">
+      <c r="F2" s="16" t="inlineStr">
         <is>
           <t>Informational</t>
         </is>
       </c>
-      <c r="G2" s="6" t="inlineStr">
-        <is>
-          <t>Global</t>
-        </is>
-      </c>
-      <c r="H2" s="6" t="n">
+      <c r="G2" s="16" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="H2" s="16" t="n">
         <v>1</v>
       </c>
+      <c r="I2" s="18" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="J2" s="19" t="inlineStr">
+        <is>
+          <t>https://saisatwik.com/what-is-sap-eppm-and-why-top-enterprises-are-switching-to-it/</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="16" t="inlineStr">
         <is>
           <t>K02</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="16" t="inlineStr">
         <is>
           <t>EPPM</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C3" s="17" t="inlineStr">
         <is>
           <t>SAP EPPM modules explained (PS, PPM, IM, CPM, CATS)</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D3" s="17" t="inlineStr">
         <is>
           <t>SAP EPPM modules</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="E3" s="17" t="inlineStr">
         <is>
           <t>SAP EPPM components, SAP EPPM suite</t>
         </is>
       </c>
-      <c r="F3" s="8" t="inlineStr">
+      <c r="F3" s="16" t="inlineStr">
         <is>
           <t>Informational</t>
         </is>
       </c>
-      <c r="G3" s="8" t="inlineStr">
-        <is>
-          <t>Global</t>
-        </is>
-      </c>
-      <c r="H3" s="8" t="n">
+      <c r="G3" s="16" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="H3" s="16" t="n">
         <v>1</v>
       </c>
+      <c r="I3" s="18" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="J3" s="19" t="inlineStr">
+        <is>
+          <t>https://saisatwik.com/sap-eppm-modules-explained-ps-ppm-im-cpm-cats/</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>K03</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="16" t="inlineStr">
         <is>
           <t>EPPM</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="17" t="inlineStr">
         <is>
           <t>SAP EPPM in SAP S/4HANA: what changed</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="D4" s="17" t="inlineStr">
         <is>
           <t>SAP EPPM S/4HANA</t>
         </is>
       </c>
-      <c r="E4" s="7" t="inlineStr">
+      <c r="E4" s="17" t="inlineStr">
         <is>
           <t>EPPM S4HANA, S/4HANA portfolio project management</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="F4" s="16" t="inlineStr">
         <is>
           <t>Informational</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>Global</t>
-        </is>
-      </c>
-      <c r="H4" s="6" t="n">
+      <c r="G4" s="16" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="H4" s="16" t="n">
         <v>1</v>
       </c>
+      <c r="I4" s="18" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="J4" s="19" t="inlineStr">
+        <is>
+          <t>https://saisatwik.com/sap-eppm-in-sap-s4hana-what-changed/</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>K04</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>EPPM</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C5" s="17" t="inlineStr">
         <is>
           <t>SAP EPPM implementation roadmap</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D5" s="17" t="inlineStr">
         <is>
           <t>SAP EPPM implementation</t>
         </is>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="E5" s="17" t="inlineStr">
         <is>
           <t>how to implement SAP EPPM, EPPM project plan</t>
         </is>
       </c>
-      <c r="F5" s="8" t="inlineStr">
+      <c r="F5" s="16" t="inlineStr">
         <is>
           <t>Informational</t>
         </is>
       </c>
-      <c r="G5" s="8" t="inlineStr">
-        <is>
-          <t>Global</t>
-        </is>
-      </c>
-      <c r="H5" s="8" t="n">
+      <c r="G5" s="16" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="H5" s="16" t="n">
         <v>2</v>
+      </c>
+      <c r="I5" s="18" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="J5" s="19" t="inlineStr">
+        <is>
+          <t>https://saisatwik.com/sap-eppm-implementation-roadmap/</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -922,6 +989,11 @@
       <c r="H6" s="6" t="n">
         <v>2</v>
       </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
@@ -962,6 +1034,11 @@
       <c r="H7" s="8" t="n">
         <v>3</v>
       </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -1002,6 +1079,11 @@
       <c r="H8" s="6" t="n">
         <v>2</v>
       </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
@@ -1042,6 +1124,11 @@
       <c r="H9" s="8" t="n">
         <v>1</v>
       </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -1082,6 +1169,11 @@
       <c r="H10" s="6" t="n">
         <v>1</v>
       </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
@@ -1122,6 +1214,11 @@
       <c r="H11" s="8" t="n">
         <v>1</v>
       </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
@@ -1162,6 +1259,11 @@
       <c r="H12" s="6" t="n">
         <v>1</v>
       </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
@@ -1202,6 +1304,11 @@
       <c r="H13" s="8" t="n">
         <v>2</v>
       </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
@@ -1242,6 +1349,11 @@
       <c r="H14" s="6" t="n">
         <v>1</v>
       </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
@@ -1282,6 +1394,11 @@
       <c r="H15" s="8" t="n">
         <v>2</v>
       </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
@@ -1322,6 +1439,11 @@
       <c r="H16" s="6" t="n">
         <v>1</v>
       </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
@@ -1362,6 +1484,11 @@
       <c r="H17" s="8" t="n">
         <v>2</v>
       </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
@@ -1402,6 +1529,11 @@
       <c r="H18" s="6" t="n">
         <v>2</v>
       </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
@@ -1442,6 +1574,11 @@
       <c r="H19" s="8" t="n">
         <v>2</v>
       </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
@@ -1482,6 +1619,11 @@
       <c r="H20" s="6" t="n">
         <v>3</v>
       </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
@@ -1522,6 +1664,11 @@
       <c r="H21" s="8" t="n">
         <v>1</v>
       </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
@@ -1562,6 +1709,11 @@
       <c r="H22" s="6" t="n">
         <v>1</v>
       </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
@@ -1602,6 +1754,11 @@
       <c r="H23" s="8" t="n">
         <v>1</v>
       </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
@@ -1642,6 +1799,11 @@
       <c r="H24" s="6" t="n">
         <v>2</v>
       </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
@@ -1682,6 +1844,11 @@
       <c r="H25" s="8" t="n">
         <v>2</v>
       </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
@@ -1722,6 +1889,11 @@
       <c r="H26" s="6" t="n">
         <v>3</v>
       </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
@@ -1762,6 +1934,11 @@
       <c r="H27" s="8" t="n">
         <v>1</v>
       </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
@@ -1802,6 +1979,11 @@
       <c r="H28" s="6" t="n">
         <v>3</v>
       </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
@@ -1842,6 +2024,11 @@
       <c r="H29" s="8" t="n">
         <v>1</v>
       </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
@@ -1882,6 +2069,11 @@
       <c r="H30" s="6" t="n">
         <v>1</v>
       </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
@@ -1922,6 +2114,11 @@
       <c r="H31" s="8" t="n">
         <v>2</v>
       </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
@@ -1962,6 +2159,11 @@
       <c r="H32" s="6" t="n">
         <v>2</v>
       </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
@@ -2002,6 +2204,11 @@
       <c r="H33" s="8" t="n">
         <v>3</v>
       </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
@@ -2042,6 +2249,11 @@
       <c r="H34" s="6" t="n">
         <v>2</v>
       </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
@@ -2082,6 +2294,11 @@
       <c r="H35" s="8" t="n">
         <v>1</v>
       </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
@@ -2122,6 +2339,11 @@
       <c r="H36" s="6" t="n">
         <v>2</v>
       </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
@@ -2162,6 +2384,11 @@
       <c r="H37" s="8" t="n">
         <v>3</v>
       </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
@@ -2202,6 +2429,11 @@
       <c r="H38" s="6" t="n">
         <v>3</v>
       </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
@@ -2242,6 +2474,11 @@
       <c r="H39" s="8" t="n">
         <v>2</v>
       </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
@@ -2282,6 +2519,11 @@
       <c r="H40" s="6" t="n">
         <v>3</v>
       </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
@@ -2322,6 +2564,11 @@
       <c r="H41" s="8" t="n">
         <v>2</v>
       </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
@@ -2362,6 +2609,11 @@
       <c r="H42" s="6" t="n">
         <v>1</v>
       </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
@@ -2402,6 +2654,11 @@
       <c r="H43" s="8" t="n">
         <v>2</v>
       </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
@@ -2442,6 +2699,11 @@
       <c r="H44" s="6" t="n">
         <v>3</v>
       </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
@@ -2482,6 +2744,11 @@
       <c r="H45" s="8" t="n">
         <v>3</v>
       </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
@@ -2522,6 +2789,11 @@
       <c r="H46" s="6" t="n">
         <v>1</v>
       </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
@@ -2562,6 +2834,11 @@
       <c r="H47" s="8" t="n">
         <v>1</v>
       </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
@@ -2602,6 +2879,11 @@
       <c r="H48" s="6" t="n">
         <v>2</v>
       </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
@@ -2642,6 +2924,11 @@
       <c r="H49" s="8" t="n">
         <v>1</v>
       </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
@@ -2682,6 +2969,11 @@
       <c r="H50" s="6" t="n">
         <v>1</v>
       </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
@@ -2722,6 +3014,11 @@
       <c r="H51" s="8" t="n">
         <v>2</v>
       </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
@@ -2762,6 +3059,11 @@
       <c r="H52" s="6" t="n">
         <v>1</v>
       </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
@@ -2802,6 +3104,11 @@
       <c r="H53" s="8" t="n">
         <v>2</v>
       </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
@@ -2842,6 +3149,11 @@
       <c r="H54" s="6" t="n">
         <v>2</v>
       </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="8" t="inlineStr">
@@ -2882,6 +3194,11 @@
       <c r="H55" s="8" t="n">
         <v>2</v>
       </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
@@ -2922,6 +3239,11 @@
       <c r="H56" s="6" t="n">
         <v>1</v>
       </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="8" t="inlineStr">
@@ -2962,6 +3284,11 @@
       <c r="H57" s="8" t="n">
         <v>1</v>
       </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
@@ -3002,6 +3329,11 @@
       <c r="H58" s="6" t="n">
         <v>1</v>
       </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="8" t="inlineStr">
@@ -3042,6 +3374,11 @@
       <c r="H59" s="8" t="n">
         <v>2</v>
       </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
@@ -3082,6 +3419,11 @@
       <c r="H60" s="6" t="n">
         <v>2</v>
       </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="8" t="inlineStr">
@@ -3122,6 +3464,11 @@
       <c r="H61" s="8" t="n">
         <v>2</v>
       </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
@@ -3162,6 +3509,11 @@
       <c r="H62" s="6" t="n">
         <v>2</v>
       </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="8" t="inlineStr">
@@ -3202,6 +3554,11 @@
       <c r="H63" s="8" t="n">
         <v>3</v>
       </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
@@ -3242,6 +3599,11 @@
       <c r="H64" s="6" t="n">
         <v>3</v>
       </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="8" t="inlineStr">
@@ -3282,45 +3644,60 @@
       <c r="H65" s="8" t="n">
         <v>3</v>
       </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="66">
-      <c r="A66" s="6" t="inlineStr">
+      <c r="A66" s="16" t="inlineStr">
         <is>
           <t>K65</t>
         </is>
       </c>
-      <c r="B66" s="6" t="inlineStr">
+      <c r="B66" s="16" t="inlineStr">
         <is>
           <t>Regional</t>
         </is>
       </c>
-      <c r="C66" s="7" t="inlineStr">
+      <c r="C66" s="17" t="inlineStr">
         <is>
           <t>SAP EPPM and Saudi Vision 2030 giga-projects</t>
         </is>
       </c>
-      <c r="D66" s="7" t="inlineStr">
+      <c r="D66" s="17" t="inlineStr">
         <is>
           <t>SAP EPPM Vision 2030</t>
         </is>
       </c>
-      <c r="E66" s="7" t="inlineStr">
+      <c r="E66" s="17" t="inlineStr">
         <is>
           <t>giga project SAP, vision 2030 project controls</t>
         </is>
       </c>
-      <c r="F66" s="6" t="inlineStr">
+      <c r="F66" s="16" t="inlineStr">
         <is>
           <t>Informational</t>
         </is>
       </c>
-      <c r="G66" s="6" t="inlineStr">
+      <c r="G66" s="16" t="inlineStr">
         <is>
           <t>KSA / Gulf</t>
         </is>
       </c>
-      <c r="H66" s="6" t="n">
+      <c r="H66" s="16" t="n">
         <v>1</v>
+      </c>
+      <c r="I66" s="18" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="J66" s="19" t="inlineStr">
+        <is>
+          <t>https://saisatwik.com/why-saudi-enterprises-are-adopting-sap-eppm-for-large-project-portfolios/</t>
+        </is>
       </c>
     </row>
     <row r="67">
@@ -3362,6 +3739,11 @@
       <c r="H67" s="8" t="n">
         <v>2</v>
       </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
@@ -3401,6 +3783,11 @@
       </c>
       <c r="H68" s="6" t="n">
         <v>3</v>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -3415,7 +3802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:J37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3426,6 +3813,8 @@
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -3469,6 +3858,16 @@
           <t>Priority</t>
         </is>
       </c>
+      <c r="I1" s="15" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="J1" s="15" t="inlineStr">
+        <is>
+          <t>Live URL</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
@@ -3509,6 +3908,11 @@
       <c r="H2" s="6" t="n">
         <v>1</v>
       </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
@@ -3549,6 +3953,11 @@
       <c r="H3" s="8" t="n">
         <v>1</v>
       </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -3589,6 +3998,11 @@
       <c r="H4" s="6" t="n">
         <v>1</v>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
@@ -3629,6 +4043,11 @@
       <c r="H5" s="8" t="n">
         <v>1</v>
       </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -3669,6 +4088,11 @@
       <c r="H6" s="6" t="n">
         <v>2</v>
       </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
@@ -3709,6 +4133,11 @@
       <c r="H7" s="8" t="n">
         <v>1</v>
       </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -3749,6 +4178,11 @@
       <c r="H8" s="6" t="n">
         <v>1</v>
       </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
@@ -3789,6 +4223,11 @@
       <c r="H9" s="8" t="n">
         <v>2</v>
       </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -3829,6 +4268,11 @@
       <c r="H10" s="6" t="n">
         <v>1</v>
       </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
@@ -3869,6 +4313,11 @@
       <c r="H11" s="8" t="n">
         <v>2</v>
       </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
@@ -3909,6 +4358,11 @@
       <c r="H12" s="6" t="n">
         <v>2</v>
       </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
@@ -3949,6 +4403,11 @@
       <c r="H13" s="8" t="n">
         <v>2</v>
       </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
@@ -3989,6 +4448,11 @@
       <c r="H14" s="6" t="n">
         <v>3</v>
       </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
@@ -4029,6 +4493,11 @@
       <c r="H15" s="8" t="n">
         <v>1</v>
       </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
@@ -4069,6 +4538,11 @@
       <c r="H16" s="6" t="n">
         <v>1</v>
       </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
@@ -4109,6 +4583,11 @@
       <c r="H17" s="8" t="n">
         <v>1</v>
       </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
@@ -4149,6 +4628,11 @@
       <c r="H18" s="6" t="n">
         <v>1</v>
       </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
@@ -4189,6 +4673,11 @@
       <c r="H19" s="8" t="n">
         <v>1</v>
       </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
@@ -4229,6 +4718,11 @@
       <c r="H20" s="6" t="n">
         <v>1</v>
       </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
@@ -4269,6 +4763,11 @@
       <c r="H21" s="8" t="n">
         <v>1</v>
       </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
@@ -4309,6 +4808,11 @@
       <c r="H22" s="6" t="n">
         <v>2</v>
       </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
@@ -4349,6 +4853,11 @@
       <c r="H23" s="8" t="n">
         <v>2</v>
       </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
@@ -4389,6 +4898,11 @@
       <c r="H24" s="6" t="n">
         <v>2</v>
       </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
@@ -4429,6 +4943,11 @@
       <c r="H25" s="8" t="n">
         <v>3</v>
       </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
@@ -4469,6 +4988,11 @@
       <c r="H26" s="6" t="n">
         <v>2</v>
       </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
@@ -4509,6 +5033,11 @@
       <c r="H27" s="8" t="n">
         <v>2</v>
       </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
@@ -4549,6 +5078,11 @@
       <c r="H28" s="6" t="n">
         <v>2</v>
       </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
@@ -4589,6 +5123,11 @@
       <c r="H29" s="8" t="n">
         <v>1</v>
       </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
@@ -4629,6 +5168,11 @@
       <c r="H30" s="6" t="n">
         <v>1</v>
       </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
@@ -4669,6 +5213,11 @@
       <c r="H31" s="8" t="n">
         <v>2</v>
       </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
@@ -4709,6 +5258,11 @@
       <c r="H32" s="6" t="n">
         <v>2</v>
       </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
@@ -4749,6 +5303,11 @@
       <c r="H33" s="8" t="n">
         <v>1</v>
       </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
@@ -4789,6 +5348,11 @@
       <c r="H34" s="6" t="n">
         <v>2</v>
       </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
@@ -4829,6 +5393,11 @@
       <c r="H35" s="8" t="n">
         <v>1</v>
       </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
@@ -4869,6 +5438,11 @@
       <c r="H36" s="6" t="n">
         <v>2</v>
       </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
@@ -4908,6 +5482,11 @@
       </c>
       <c r="H37" s="8" t="n">
         <v>1</v>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -5705,8 +6284,6 @@
           <t>How to use</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr"/>
-      <c r="C1" t="inlineStr"/>
     </row>
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="11" t="inlineStr">

</xml_diff>

<commit_message>
feat(saisatwik): publish K05 (SAP EPPM architecture + integration), spoke #9; mark workbook
</commit_message>
<xml_diff>
--- a/SAP-EPPM-PS-Blog-Keyword-Plan.xlsx
+++ b/SAP-EPPM-PS-Blog-Keyword-Plan.xlsx
@@ -558,7 +558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="B1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -951,47 +951,52 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>K05</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="16" t="inlineStr">
         <is>
           <t>EPPM</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="17" t="inlineStr">
         <is>
           <t>SAP EPPM architecture and integration overview</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="17" t="inlineStr">
         <is>
           <t>SAP EPPM architecture</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="E6" s="17" t="inlineStr">
         <is>
           <t>EPPM integration, EPPM landscape</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="F6" s="16" t="inlineStr">
         <is>
           <t>Informational</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>Global</t>
-        </is>
-      </c>
-      <c r="H6" s="6" t="n">
+      <c r="G6" s="16" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="H6" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I6" s="18" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="J6" s="19" t="inlineStr">
+        <is>
+          <t>https://saisatwik.com/sap-eppm-architecture-and-integration-overview/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(saisatwik): publish K06 (SAP EPPM licensing), spoke #10; mark workbook
</commit_message>
<xml_diff>
--- a/SAP-EPPM-PS-Blog-Keyword-Plan.xlsx
+++ b/SAP-EPPM-PS-Blog-Keyword-Plan.xlsx
@@ -1001,47 +1001,52 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>K06</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="16" t="inlineStr">
         <is>
           <t>EPPM</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="17" t="inlineStr">
         <is>
           <t>SAP EPPM licensing explained</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D7" s="17" t="inlineStr">
         <is>
           <t>SAP EPPM licensing</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="E7" s="17" t="inlineStr">
         <is>
           <t>SAP EPPM cost, EPPM license types</t>
         </is>
       </c>
-      <c r="F7" s="8" t="inlineStr">
+      <c r="F7" s="16" t="inlineStr">
         <is>
           <t>Informational</t>
         </is>
       </c>
-      <c r="G7" s="8" t="inlineStr">
-        <is>
-          <t>Global</t>
-        </is>
-      </c>
-      <c r="H7" s="8" t="n">
+      <c r="G7" s="16" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="H7" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I7" s="18" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="J7" s="19" t="inlineStr">
+        <is>
+          <t>https://saisatwik.com/sap-eppm-licensing-explained/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: mark K07 published in workbook
</commit_message>
<xml_diff>
--- a/SAP-EPPM-PS-Blog-Keyword-Plan.xlsx
+++ b/SAP-EPPM-PS-Blog-Keyword-Plan.xlsx
@@ -1051,47 +1051,52 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>K07</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="16" t="inlineStr">
         <is>
           <t>EPPM</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="17" t="inlineStr">
         <is>
           <t>SAP EPPM best practices for capital projects</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D8" s="17" t="inlineStr">
         <is>
           <t>SAP EPPM best practices</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="E8" s="17" t="inlineStr">
         <is>
           <t>capital project management SAP</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="F8" s="16" t="inlineStr">
         <is>
           <t>Informational</t>
         </is>
       </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>Global</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="n">
+      <c r="G8" s="16" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="H8" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I8" s="18" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="J8" s="19" t="inlineStr">
+        <is>
+          <t>https://saisatwik.com/sap-eppm-best-practices-for-capital-projects/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(saisatwik): publish K08 (What is SAP PS) - opens SAP PS cluster hub; mark workbook
</commit_message>
<xml_diff>
--- a/SAP-EPPM-PS-Blog-Keyword-Plan.xlsx
+++ b/SAP-EPPM-PS-Blog-Keyword-Plan.xlsx
@@ -1101,47 +1101,52 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>K08</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="16" t="inlineStr">
         <is>
           <t>SAP PS</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="17" t="inlineStr">
         <is>
           <t>What is SAP PS (Project System)? Beginner guide</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D9" s="17" t="inlineStr">
         <is>
           <t>what is SAP PS module</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="E9" s="17" t="inlineStr">
         <is>
           <t>SAP PS meaning, SAP Project System overview</t>
         </is>
       </c>
-      <c r="F9" s="8" t="inlineStr">
+      <c r="F9" s="16" t="inlineStr">
         <is>
           <t>Informational</t>
         </is>
       </c>
-      <c r="G9" s="8" t="inlineStr">
-        <is>
-          <t>Global</t>
-        </is>
-      </c>
-      <c r="H9" s="8" t="n">
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I9" s="18" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="J9" s="19" t="inlineStr">
+        <is>
+          <t>https://saisatwik.com/what-is-sap-ps-project-system-beginner-guide/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content(saisatwik): publish K09 SAP PS tutorial for beginners (#5423)
- New spoke of the SAP PS cluster under hub #5418: six-step lifecycle
  tutorial (CJ20N structure -> networks -> CJ40 planning -> CJ30/CJ32
  budget -> actuals -> CJI3/CJ88 monitor+settle), 10-tcode table,
  learning-path table, 5-question FAQ, 3 outbound authority links
  (SAP Help Portal, SAP Learning, sap.com), 9 internal links
- Hub #5418 re-pushed with the tutorial linked from Related Reading and
  the learn-SAP-PS FAQ
- TAGS.md: registered SAP PS (Technology) + Tutorial (Format)
- CLUSTERS.md: K09 marked live; workbook row K09 marked Published+green

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SAP-EPPM-PS-Blog-Keyword-Plan.xlsx
+++ b/SAP-EPPM-PS-Blog-Keyword-Plan.xlsx
@@ -1151,47 +1151,52 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>K09</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="16" t="inlineStr">
         <is>
           <t>SAP PS</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="17" t="inlineStr">
         <is>
           <t>SAP PS tutorial for beginners</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D10" s="17" t="inlineStr">
         <is>
           <t>SAP PS tutorial</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="E10" s="17" t="inlineStr">
         <is>
           <t>SAP PS training, learn SAP PS, SAP PS step by step</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="F10" s="16" t="inlineStr">
         <is>
           <t>Informational</t>
         </is>
       </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>Global</t>
-        </is>
-      </c>
-      <c r="H10" s="6" t="n">
+      <c r="G10" s="16" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="H10" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I10" s="19" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="J10" s="19" t="inlineStr">
+        <is>
+          <t>https://saisatwik.com/sap-ps-tutorial-for-beginners/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content(saisatwik): publish K10 SAP PS WBS explained (#5425)
- Third post of the SAP PS cluster: WBS deep dive with the three
  operative indicators table, CJ20N creation steps, level-count
  guidance, 5-rule design table, cost-control chain (CJ40 -> CJ30/CJ32
  -> availability control -> CJ88), 5-question FAQ incl. coding mask
  and SAP-vs-Primavera WBS
- Outbound: PMI, SAP Help Portal, sap.com. 9 internal links.
- Hub #5418 and tutorial #5423 re-pushed with WBS guide cross-links
  (hub Related Reading + tutorial Step 1 operative-indicators anchor)
- CLUSTERS.md K10 live; workbook K10 Published + green; new WP tag
  "Engineering and Construction" (#78) already registered in TAGS.md

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SAP-EPPM-PS-Blog-Keyword-Plan.xlsx
+++ b/SAP-EPPM-PS-Blog-Keyword-Plan.xlsx
@@ -1201,47 +1201,52 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>K10</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="16" t="inlineStr">
         <is>
           <t>SAP PS</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C11" s="17" t="inlineStr">
         <is>
           <t>SAP PS Work Breakdown Structure (WBS) explained</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D11" s="17" t="inlineStr">
         <is>
           <t>SAP PS WBS</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr">
+      <c r="E11" s="17" t="inlineStr">
         <is>
           <t>WBS element SAP, create WBS SAP PS</t>
         </is>
       </c>
-      <c r="F11" s="8" t="inlineStr">
+      <c r="F11" s="16" t="inlineStr">
         <is>
           <t>Informational</t>
         </is>
       </c>
-      <c r="G11" s="8" t="inlineStr">
-        <is>
-          <t>Global</t>
-        </is>
-      </c>
-      <c r="H11" s="8" t="n">
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I11" s="19" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="J11" s="19" t="inlineStr">
+        <is>
+          <t>https://saisatwik.com/sap-ps-work-breakdown-structure-wbs-explained/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
content(saisatwik): publish K11 CJ20N project creation guide (#5428)
- Fourth SAP PS cluster post: Project Builder how-to. Quick Answer,
  CJ20N vs legacy CJ01/CJ02/CN21 context, prerequisites, 5 creation
  steps (definition -> WBS -> networks/milestones -> scheduling ->
  release), 6-row common-errors table (coding mask, CRTD block, AA
  indicator, availability control, deletion, locks), practitioner
  shortcuts (templates, worklist, inheritance), 5 FAQs
- Outbound: sap.com S/4HANA, SAP Help Portal, SAP Learning. 8 internal.
- Cross-links re-pushed: hub #5418 Related Reading, tutorial #5423
  Step 1, WBS guide #5425 creation section
- CLUSTERS.md K11 live; workbook K11 Published + green

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SAP-EPPM-PS-Blog-Keyword-Plan.xlsx
+++ b/SAP-EPPM-PS-Blog-Keyword-Plan.xlsx
@@ -1251,47 +1251,52 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="16" t="inlineStr">
         <is>
           <t>K11</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="16" t="inlineStr">
         <is>
           <t>SAP PS</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="17" t="inlineStr">
         <is>
           <t>How to create a project in SAP PS (CJ20N)</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D12" s="17" t="inlineStr">
         <is>
           <t>CJ20N SAP PS</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="E12" s="17" t="inlineStr">
         <is>
           <t>project builder SAP, CJ20N tutorial</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="F12" s="16" t="inlineStr">
         <is>
           <t>Informational</t>
         </is>
       </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>Global</t>
-        </is>
-      </c>
-      <c r="H12" s="6" t="n">
+      <c r="G12" s="16" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="H12" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>Pending</t>
+      <c r="I12" s="19" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="J12" s="19" t="inlineStr">
+        <is>
+          <t>https://saisatwik.com/how-to-create-a-project-in-sap-ps-cj20n/</t>
         </is>
       </c>
     </row>

</xml_diff>